<commit_message>
NS: changed promrotores to fit with alon kahani estimates
</commit_message>
<xml_diff>
--- a/background_files/promoteres.xlsx
+++ b/background_files/promoteres.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Data\Forecast\Tools\forecast_git\create_forecast_ad_hoc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\background_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C421B0-C4A3-4130-ABB7-F7B4378EA3E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B840BA-655A-4469-967B-3FBCF1C20586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -526,7 +526,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>200</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -534,7 +534,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -542,7 +542,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -550,7 +550,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>60</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed promoter of student per education to 9
</commit_message>
<xml_diff>
--- a/background_files/promoteres.xlsx
+++ b/background_files/promoteres.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\background_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\background_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B840BA-655A-4469-967B-3FBCF1C20586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87681A9B-96F2-4F5A-87DB-583D6883DFCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -459,13 +459,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="34.21875" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" customWidth="1"/>
+    <col min="1" max="1" width="34.28515625" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -473,7 +473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -481,7 +481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -489,7 +489,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -497,7 +497,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -505,7 +505,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -513,7 +513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -521,7 +521,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -529,7 +529,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -537,7 +537,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -545,7 +545,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -553,7 +553,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -561,7 +561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -569,7 +569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -577,7 +577,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -585,7 +585,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -593,7 +593,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -601,15 +601,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>18</v>
       </c>
       <c r="B18">
-        <v>3.75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -617,7 +617,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
adding promoters to for approvel + changing names to heb+adding description in promoters file - still need to complete
</commit_message>
<xml_diff>
--- a/background_files/promoteres.xlsx
+++ b/background_files/promoteres.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\background_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87681A9B-96F2-4F5A-87DB-583D6883DFCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A796FED-CC0B-41E2-9119-D24D4A9D3DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
   <si>
     <t>key</t>
   </si>
@@ -88,18 +88,62 @@
   </si>
   <si>
     <t>emp_Education_per_Yeshiva_student</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description </t>
+  </si>
+  <si>
+    <t>חישוב מועסקים ממ"ר תעשייה - מועסק על כל 100 מ"ר</t>
+  </si>
+  <si>
+    <t>חישוב מועסקים ממ"ר מסחר ומלונאות - מועסק על כל 50 מ"ר</t>
+  </si>
+  <si>
+    <t>חישוב מועסקים ממ"ר תעסוקה (משרדים) - מועסק על כל 50 מ"ר</t>
+  </si>
+  <si>
+    <t>חישוב מועסקים ממ"ר ציבורי - מועסק על כל 20 מ"ר</t>
+  </si>
+  <si>
+    <t>חישוב מועסקים מחקלאות - 0 קבוע</t>
+  </si>
+  <si>
+    <t>חישוב מועסקים ממ"ר חינוך - 0 קבוע, שימו לב כי מועסקים בחינוך מחושבים לפי תלמידים</t>
+  </si>
+  <si>
+    <t>חישוב מועסקים ממ"ר תיירות - מועסק על כל 100 מ"ר</t>
+  </si>
+  <si>
+    <t xml:space="preserve">חישוב מועסקי חינוך מתלמידים - איש צוות על כל 9 תלמידים </t>
+  </si>
+  <si>
+    <t>חישוב מועסקי חינוך מסטודנטים - איש צוות על כל 10 סטודנטים 
+(*שימו לב* - מקדם זה מוכפל בנתון ולא מחולק בו.)</t>
+  </si>
+  <si>
+    <t>חישוב מועסקי חינוך מתלמידי ישיבו - איש צוות על כל 10 סטודנטים 
+(*שימו לב* - מקדם זה מוכפל בנתון ולא מחולק בו.)</t>
+  </si>
+  <si>
+    <t>לא ידעתי להסביר</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -122,8 +166,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -458,175 +506,236 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultColWidth="12.7265625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.28515625" customWidth="1"/>
-    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="1" max="1" width="34.26953125" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" customWidth="1"/>
+    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C3" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C5" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C7" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8">
         <v>100</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
       <c r="B9">
         <v>50</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
       <c r="B11">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
       <c r="B12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="25" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C13" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C14" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
       <c r="B15">
         <v>100</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
       <c r="B16">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C16" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
       <c r="B17">
         <v>3</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C17" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
       <c r="B18">
         <v>9</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
       <c r="B19">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C19" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
       <c r="B20">
         <v>0.1</v>
       </c>
+      <c r="C20" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
adding plans, zip, new sheet and explanation file
</commit_message>
<xml_diff>
--- a/background_files/promoteres.xlsx
+++ b/background_files/promoteres.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\background_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A796FED-CC0B-41E2-9119-D24D4A9D3DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A09F39D-F2FB-4E8C-B595-F84DEE13060E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>key</t>
   </si>
@@ -125,14 +125,17 @@
 (*שימו לב* - מקדם זה מוכפל בנתון ולא מחולק בו.)</t>
   </si>
   <si>
-    <t>לא ידעתי להסביר</t>
+    <t>כל 1.5 אנשים בבית אבות נחשבים משק בית אחד</t>
+  </si>
+  <si>
+    <t>כל 3 אנשים במעונות נחשבים משק בית אחד</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -142,6 +145,11 @@
     <font>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -166,12 +174,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,9 +541,7 @@
       <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -543,9 +550,7 @@
       <c r="B3">
         <v>0.55000000000000004</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -554,9 +559,7 @@
       <c r="B4">
         <v>0.2</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -565,9 +568,7 @@
       <c r="B5">
         <v>0.25</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -576,9 +577,7 @@
       <c r="B6">
         <v>0</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -587,9 +586,7 @@
       <c r="B7">
         <v>0.1</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -664,9 +661,7 @@
       <c r="B14" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -686,7 +681,7 @@
       <c r="B16">
         <v>1.5</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>32</v>
       </c>
     </row>
@@ -697,8 +692,8 @@
       <c r="B17">
         <v>3</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>32</v>
+      <c r="C17" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>